<commit_message>
Propuestas de nombre y descripción para 39 productos (en borrador)
13 de piel (fichas oficiales o empaque) y 26 de bienestar íntimo (empaque),
con nombres corregidos o neutralizados y precauciones. Quedan en estado
"borrador" hasta que Diana los apruebe; la fuente de cada texto está en
notas_internas. El sitio publicado no cambia (122 productos).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/catalogo.xlsx
+++ b/catalogo/catalogo.xlsx
@@ -15881,16 +15881,20 @@
       </c>
     </row>
     <row r="120" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A120" s="6" t="s">
-        <v>56</v>
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-015</t>
         </is>
       </c>
-      <c r="C120" t="s">
-        <v>1641</v>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Sunface Aqua Antipigment</t>
+        </is>
       </c>
       <c r="D120" s="6" t="s">
         <v>1625</v>
@@ -15905,10 +15909,40 @@
       <c r="J120" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Fotoprotector facial SPF 50+ sin color, de textura ligera y acabado sedoso, que ayuda a prevenir la aparición de manchas.</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Piel mixta.</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Aplicar sobre rostro, cuello y manos 30 minutos antes de la exposición solar. Reaplicar cada 3 horas o después de sudar, nadar o secarse con toalla.</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>60 g</t>
+        </is>
+      </c>
       <c r="AC120" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-015/</v>
       </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: ficha oficial https://skindrug.com.co/producto/sunface-aqua-antipigment/ y empaque. Aviso: El nombre del Excel decía "Aqua sin color"; el empaque y la ficha oficial dicen "Aqua Antipigment".</t>
+        </is>
+      </c>
     </row>
     <row r="121" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A121" s="6" t="s">
@@ -16525,16 +16559,20 @@
       </c>
     </row>
     <row r="131" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A131" s="6" t="s">
-        <v>56</v>
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-026</t>
         </is>
       </c>
-      <c r="C131" t="s">
-        <v>1652</v>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Sunstop Oil Free Color</t>
+        </is>
       </c>
       <c r="D131" s="6" t="s">
         <v>106</v>
@@ -16549,10 +16587,35 @@
       <c r="J131" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Fotoprotector SPF 50+ con color, de toque seco y acabado matificado, que ayuda a unificar el tono. Puede reemplazar la base de maquillaje.</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Piel mixta a grasa.</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>Aplicar sobre rostro, orejas, cuello y manos 30 minutos antes de la exposición solar. Reaplicar cada 3 horas o después de sudar, nadar o limpiar la piel.</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC131" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-026/</v>
       </c>
+      <c r="AG131" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: ficha oficial https://pharmaderm.com.co/producto/sunstop-oil-free-color/ y empaque. Aviso: Es el mismo producto que ESZ-PIE-001 (SunStop Oil Free Color, en borrador y sin precio). Conviene dejar solo uno.</t>
+        </is>
+      </c>
     </row>
     <row r="132" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A132" s="6" t="s">
@@ -16745,16 +16808,20 @@
       </c>
     </row>
     <row r="135" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A135" s="6" t="s">
-        <v>56</v>
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-030</t>
         </is>
       </c>
-      <c r="C135" t="s">
-        <v>1656</v>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Hydraxer Lifting Effect ampollas</t>
+        </is>
       </c>
       <c r="D135" s="6" t="s">
         <v>1707</v>
@@ -16769,22 +16836,41 @@
       <c r="J135" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Ampollas anti-edad Hydraxer Lifting Effect de DermaElite, con efecto tensor e hidratante. Paso 3 de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC135" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-030/</v>
       </c>
+      <c r="AG135" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="136" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A136" s="6" t="s">
-        <v>56</v>
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-031</t>
         </is>
       </c>
-      <c r="C136" t="s">
-        <v>1657</v>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Hydraxer Aqua agua micelar</t>
+        </is>
       </c>
       <c r="D136" s="6" t="s">
         <v>1707</v>
@@ -16799,22 +16885,41 @@
       <c r="J136" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Agua micelar hialurónica de DermaElite que limpia y desmaquilla mientras ayuda a mantener la hidratación. Paso 1 de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC136" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-031/</v>
       </c>
+      <c r="AG136" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="137" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A137" s="6" t="s">
-        <v>56</v>
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-032</t>
         </is>
       </c>
-      <c r="C137" t="s">
-        <v>1658</v>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Hydraxer Eyes contorno de ojos</t>
+        </is>
       </c>
       <c r="D137" s="6" t="s">
         <v>1707</v>
@@ -16829,22 +16934,46 @@
       <c r="J137" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Contorno de ojos Hydraxer Eyes de DermaElite, para el cuidado diario de la piel alrededor de los ojos. Paso 2 de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>30 g</t>
+        </is>
+      </c>
       <c r="AC137" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-032/</v>
       </c>
+      <c r="AG137" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="138" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A138" s="6" t="s">
-        <v>56</v>
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-033</t>
         </is>
       </c>
-      <c r="C138" t="s">
-        <v>1659</v>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Hydraxer Filling redensificador facial</t>
+        </is>
       </c>
       <c r="D138" s="6" t="s">
         <v>1707</v>
@@ -16859,22 +16988,46 @@
       <c r="J138" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Redensificador facial Hydraxer Filling con efecto relleno, que ayuda a hidratar y a prevenir las arrugas profundas. Paso 3 de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>30 g</t>
+        </is>
+      </c>
       <c r="AC138" s="6" t="str">
         <f t="shared" si="0"/>
         <v>productos/ESZ-PIE-033/</v>
       </c>
+      <c r="AG138" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="139" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A139" s="6" t="s">
-        <v>56</v>
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-034</t>
         </is>
       </c>
-      <c r="C139" t="s">
-        <v>1660</v>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Hydraxer Face Oil Free hidratante facial</t>
+        </is>
       </c>
       <c r="D139" s="6" t="s">
         <v>1707</v>
@@ -16889,22 +17042,41 @@
       <c r="J139" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Hidratante facial Hydraxer Face Oil Free de DermaElite, libre de aceites y de hidratación prolongada. Paso 4 de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC139" s="6" t="str">
         <f t="shared" ref="AC139:AC169" si="1">IF(B139="","","productos/"&amp;B139&amp;"/")</f>
         <v>productos/ESZ-PIE-034/</v>
       </c>
+      <c r="AG139" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Hydaxer Hidratante colágeno"; el empaque dice "Hydraxer Face Oil Free · Hidratante facial" y no menciona colágeno.</t>
+        </is>
+      </c>
     </row>
     <row r="140" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A140" s="6" t="s">
-        <v>56</v>
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-035</t>
         </is>
       </c>
-      <c r="C140" t="s">
-        <v>1661</v>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Hydraxer Fluid fotoprotector SPF 50+</t>
+        </is>
       </c>
       <c r="D140" s="6" t="s">
         <v>1707</v>
@@ -16919,22 +17091,41 @@
       <c r="J140" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Fotoprotector facial SPF 50+ Hydraxer Fluid de DermaElite, de textura fluida, con OTZ 10. Paso 5 y final de la rutina Hydraxer.</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC140" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-035/</v>
       </c>
+      <c r="AG140" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="141" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A141" s="6" t="s">
-        <v>56</v>
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-036</t>
         </is>
       </c>
-      <c r="C141" t="s">
-        <v>1662</v>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Hydraxer Hyaluron Booster</t>
+        </is>
       </c>
       <c r="D141" s="6" t="s">
         <v>1707</v>
@@ -16949,22 +17140,41 @@
       <c r="J141" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Sérum Hydraxer Hyaluron Booster de DermaElite, voluminizador con ácido hialurónico y probióticos que ayuda a hidratar la piel del rostro.</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
       <c r="AC141" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-036/</v>
       </c>
+      <c r="AG141" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="142" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A142" s="6" t="s">
-        <v>56</v>
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-037</t>
         </is>
       </c>
-      <c r="C142" t="s">
-        <v>1663</v>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>MEE protector solar Oil Free SPF 50</t>
+        </is>
       </c>
       <c r="D142" s="6" t="s">
         <v>1708</v>
@@ -16979,22 +17189,46 @@
       <c r="J142" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Protector solar oil free SPF 50 de MEE, con protección UVA, UVB y luz azul, que ayuda a controlar el exceso de grasa. Tubo de 120 g.</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>120 g</t>
+        </is>
+      </c>
       <c r="AC142" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-037/</v>
       </c>
+      <c r="AG142" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+        </is>
+      </c>
     </row>
     <row r="143" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A143" s="6" t="s">
-        <v>56</v>
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-038</t>
         </is>
       </c>
-      <c r="C143" t="s">
-        <v>1664</v>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Repaskin Invisible SPF 50+</t>
+        </is>
       </c>
       <c r="D143" s="6" t="s">
         <v>1709</v>
@@ -17009,22 +17243,46 @@
       <c r="J143" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Fotoprotector facial Sesderma Repaskin Invisible SPF 50+, de textura fluida ultraligera que se absorbe rápido y no deja rastro blanco.</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
       <c r="AC143" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-038/</v>
       </c>
+      <c r="AG143" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque y fichas de distribuidores autorizados de Sesderma.</t>
+        </is>
+      </c>
     </row>
     <row r="144" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A144" s="6" t="s">
-        <v>56</v>
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-039</t>
         </is>
       </c>
-      <c r="C144" t="s">
-        <v>1665</v>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Cetopic crema con vitamina C</t>
+        </is>
       </c>
       <c r="D144" s="6" t="s">
         <v>1710</v>
@@ -17039,22 +17297,56 @@
       <c r="J144" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Crema facial con vitamina C, ácido hialurónico y pantenol, para el cuidado diario del rostro, el cuello y el contorno de ojos.</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Sodium ascorbyl phosphate, sodium hyaluronate, glycolic acid, tocopheryl acetate, panthenol.</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>Aplicar sobre la piel limpia del contorno de ojos, el rostro y el cuello, en la mañana y en la noche.</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>50 g</t>
+        </is>
+      </c>
       <c r="AC144" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-039/</v>
       </c>
+      <c r="AG144" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque y ficha técnica PLM https://www.medicamentosplm.com/Home/productos/cetopic_crema/83/101/51564/36.</t>
+        </is>
+      </c>
     </row>
     <row r="145" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="6" t="s">
-        <v>56</v>
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
           <t>ESZ-PIE-040</t>
         </is>
       </c>
-      <c r="C145" t="s">
-        <v>1666</v>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Lign-D sérum para líneas de expresión</t>
+        </is>
       </c>
       <c r="D145" s="6" t="s">
         <v>1711</v>
@@ -17069,10 +17361,30 @@
       <c r="J145" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Sérum Lign-D de Saderma para las líneas de expresión, con efecto lifting, antioxidante e hidratante. Frasco gotero de 30 ml.</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Uso externo. Evita el contacto con los ojos. Si notas irritación, suspende su uso y consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
       <c r="AC145" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-PIE-040/</v>
       </c>
+      <c r="AG145" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Ling-D"; el empaque dice "Lign-D".</t>
+        </is>
+      </c>
     </row>
     <row r="146" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A146" s="6" t="s">
@@ -17422,16 +17734,20 @@
       </c>
     </row>
     <row r="156" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A156" s="6" t="s">
-        <v>56</v>
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B156" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-105</t>
         </is>
       </c>
-      <c r="C156" s="6" t="s">
-        <v>1731</v>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>Shilajit resina del Himalaya 100 g</t>
+        </is>
       </c>
       <c r="D156" s="6" t="s">
         <v>85</v>
@@ -17448,6 +17764,21 @@
       <c r="J156" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Resina de shilajit del Himalaya en frasco de 100 g. Es un suplemento, no un medicamento; consulta a un profesional de la salud antes de usarlo.</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>No es un medicamento. Consulta a un profesional de la salud antes de usarlo, sobre todo si estás en embarazo, lactancia o tomas medicamentos.</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>100 g</t>
+        </is>
+      </c>
       <c r="Y156" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17457,18 +17788,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-105/</v>
       </c>
+      <c r="AG156" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Es un suplemento clasificado en Bienestar íntimo. El empaque dice a la vez "Ointment" (ungüento) y "Dietary supplement": confirma cómo se usa y su registro INVIMA.</t>
+        </is>
+      </c>
     </row>
     <row r="157" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A157" s="6" t="s">
-        <v>56</v>
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B157" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-106</t>
         </is>
       </c>
-      <c r="C157" s="6" t="s">
-        <v>1733</v>
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>Rozino Love bálsamo sólido en barra</t>
+        </is>
       </c>
       <c r="D157" s="6" t="s">
         <v>85</v>
@@ -17485,6 +17825,16 @@
       <c r="J157" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Bálsamo sólido perfumado Rozino Love en barra, de aplicación fácil y práctico para llevar en el bolso.</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y157" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17494,18 +17844,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-106/</v>
       </c>
+      <c r="AG157" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="158" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A158" s="6" t="s">
-        <v>56</v>
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B158" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-107</t>
         </is>
       </c>
-      <c r="C158" s="6" t="s">
-        <v>1736</v>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>Hanboli crema corporal perfumada</t>
+        </is>
       </c>
       <c r="D158" s="6" t="s">
         <v>85</v>
@@ -17520,6 +17879,16 @@
       <c r="J158" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Crema corporal perfumada Hanboli en presentación compacta, para llevar una fragancia suave contigo.</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y158" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17529,18 +17898,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-107/</v>
       </c>
+      <c r="AG158" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: El Excel decía "Hamboli"; el empaque dice "Hanboli".</t>
+        </is>
+      </c>
     </row>
     <row r="159" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A159" s="6" t="s">
-        <v>56</v>
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B159" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-108</t>
         </is>
       </c>
-      <c r="C159" s="6" t="s">
-        <v>1738</v>
+      <c r="C159" s="6" t="inlineStr">
+        <is>
+          <t>Hanboli bálsamo sólido</t>
+        </is>
       </c>
       <c r="D159" s="6" t="s">
         <v>85</v>
@@ -17555,6 +17933,16 @@
       <c r="J159" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Bálsamo sólido Hanboli en barra, de textura suave y fácil de aplicar.</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y159" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17564,18 +17952,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-108/</v>
       </c>
+      <c r="AG159" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "palpitante" del nombre: describe un efecto que no se puede verificar.</t>
+        </is>
+      </c>
     </row>
     <row r="160" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A160" s="6" t="s">
-        <v>56</v>
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B160" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-109</t>
         </is>
       </c>
-      <c r="C160" s="6" t="s">
-        <v>1740</v>
+      <c r="C160" s="6" t="inlineStr">
+        <is>
+          <t>Super Viga crema para hombre 15 ml</t>
+        </is>
       </c>
       <c r="D160" s="6" t="s">
         <v>85</v>
@@ -17590,6 +17987,21 @@
       <c r="J160" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Crema Super Viga para hombre en tubo de 15 ml. Lee las indicaciones del empaque antes de usarla.</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>15 ml</t>
+        </is>
+      </c>
       <c r="Y160" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17599,18 +18011,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-109/</v>
       </c>
+      <c r="AG160" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Es una crema retardante ("delay cream"); suelen llevar anestésico local. Confirma su registro INVIMA antes de publicarla.</t>
+        </is>
+      </c>
     </row>
     <row r="161" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A161" s="6" t="s">
-        <v>56</v>
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B161" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-110</t>
         </is>
       </c>
-      <c r="C161" s="6" t="s">
-        <v>1741</v>
+      <c r="C161" s="6" t="inlineStr">
+        <is>
+          <t>Perlas de aceite para masaje</t>
+        </is>
       </c>
       <c r="D161" s="6" t="s">
         <v>85</v>
@@ -17625,6 +18046,16 @@
       <c r="J161" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Perlas de aceite corporal para masaje, de colores, en empaque de varias unidades.</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y161" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17634,18 +18065,27 @@
         <f>IF(#REF!="","","productos/"&amp;#REF!&amp;"/")</f>
         <v>productos/ESZ-INT-110/</v>
       </c>
+      <c r="AG161" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="162" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A162" s="6" t="s">
-        <v>56</v>
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B162" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-111</t>
         </is>
       </c>
-      <c r="C162" s="6" t="s">
-        <v>1744</v>
+      <c r="C162" s="6" t="inlineStr">
+        <is>
+          <t>Ball Exotic</t>
+        </is>
       </c>
       <c r="D162" s="6" t="s">
         <v>85</v>
@@ -17660,6 +18100,11 @@
       <c r="J162" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y162" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17669,18 +18114,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-111/</v>
       </c>
+      <c r="AG162" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Con el empaque no se puede saber qué es ni cómo se usa. Diana debe escribir la descripción. Quité "anal" del nombre.</t>
+        </is>
+      </c>
     </row>
     <row r="163" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A163" s="6" t="s">
-        <v>56</v>
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B163" s="6" t="inlineStr">
         <is>
           <t>ESZ-INT-112</t>
         </is>
       </c>
-      <c r="C163" s="6" t="s">
-        <v>1745</v>
+      <c r="C163" s="6" t="inlineStr">
+        <is>
+          <t>Dados para parejas Paxion</t>
+        </is>
       </c>
       <c r="D163" s="6" t="s">
         <v>85</v>
@@ -17695,6 +18149,16 @@
       <c r="J163" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Par de dados Paxion para inventar juegos en pareja de forma divertida y sin presiones.</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y163" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17704,6 +18168,11 @@
         <f>IF(B163="","","productos/"&amp;B163&amp;"/")</f>
         <v>productos/ESZ-INT-112/</v>
       </c>
+      <c r="AG163" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="164" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="6" t="inlineStr">
@@ -17823,16 +18292,20 @@
       </c>
     </row>
     <row r="167" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A167" s="6" t="s">
-        <v>56</v>
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B167" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-116</t>
         </is>
       </c>
-      <c r="C167" s="6" t="s">
-        <v>1754</v>
+      <c r="C167" s="6" t="inlineStr">
+        <is>
+          <t>Dulce efervescente Blow Pop · Mora azul</t>
+        </is>
       </c>
       <c r="D167" s="10" t="s">
         <v>85</v>
@@ -17844,6 +18317,21 @@
         <v>10000</v>
       </c>
       <c r="I167" s="7"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Dulce efervescente Blow Pop de Elixir con sabor a mora azul, en sobre de 5 g, para sumar sabor a los momentos en pareja.</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>Contiene azúcar.</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>5 g</t>
+        </is>
+      </c>
       <c r="Y167" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17853,18 +18341,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-116/</v>
       </c>
+      <c r="AG167" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
+        </is>
+      </c>
     </row>
     <row r="168" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A168" s="6" t="s">
-        <v>56</v>
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B168" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-117</t>
         </is>
       </c>
-      <c r="C168" s="6" t="s">
-        <v>1755</v>
+      <c r="C168" s="6" t="inlineStr">
+        <is>
+          <t>Dulce efervescente Blow Pop · Sandía</t>
+        </is>
       </c>
       <c r="D168" s="10" t="s">
         <v>85</v>
@@ -17876,6 +18373,21 @@
         <v>10000</v>
       </c>
       <c r="I168" s="7"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Dulce efervescente Blow Pop de Elixir con sabor a sandía, en sobre de 5 g, para sumar sabor a los momentos en pareja.</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>Contiene azúcar.</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>5 g</t>
+        </is>
+      </c>
       <c r="Y168" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17885,18 +18397,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-117/</v>
       </c>
+      <c r="AG168" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
+        </is>
+      </c>
     </row>
     <row r="169" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A169" s="6" t="s">
-        <v>56</v>
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B169" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-118</t>
         </is>
       </c>
-      <c r="C169" s="6" t="s">
-        <v>1757</v>
+      <c r="C169" s="6" t="inlineStr">
+        <is>
+          <t>Aceite de masaje caliente · Aguardiente 80 ml</t>
+        </is>
       </c>
       <c r="D169" s="10" t="s">
         <v>85</v>
@@ -17908,6 +18429,21 @@
         <v>20000</v>
       </c>
       <c r="I169" s="7"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Aceite para masajes con sensación de calor y sabor a aguardiente, en frasco de 80 ml.</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>80 ml</t>
+        </is>
+      </c>
       <c r="Y169" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17917,18 +18453,27 @@
         <f t="shared" si="1"/>
         <v>productos/ESZ-INT-118/</v>
       </c>
+      <c r="AG169" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="170" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A170" s="6" t="s">
-        <v>56</v>
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B170" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-119</t>
         </is>
       </c>
-      <c r="C170" s="6" t="s">
-        <v>1760</v>
+      <c r="C170" s="6" t="inlineStr">
+        <is>
+          <t>Aceite de masaje caliente · Baileys 80 ml</t>
+        </is>
       </c>
       <c r="D170" s="10" t="s">
         <v>85</v>
@@ -17940,6 +18485,21 @@
         <v>20000</v>
       </c>
       <c r="I170" s="7"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Aceite para masajes con sensación de calor y sabor a crema de whisky tipo Baileys, en frasco de 80 ml.</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>80 ml</t>
+        </is>
+      </c>
       <c r="Y170" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17949,18 +18509,27 @@
         <f>IF(B170="","","productos/"&amp;B170&amp;"/")</f>
         <v>productos/ESZ-INT-119/</v>
       </c>
+      <c r="AG170" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="171" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A171" s="6" t="s">
-        <v>56</v>
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B171" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-120</t>
         </is>
       </c>
-      <c r="C171" s="6" t="s">
-        <v>1762</v>
+      <c r="C171" s="6" t="inlineStr">
+        <is>
+          <t>Aceite de masaje caliente · Ron 80 ml</t>
+        </is>
       </c>
       <c r="D171" s="10" t="s">
         <v>85</v>
@@ -17972,6 +18541,21 @@
         <v>20000</v>
       </c>
       <c r="I171" s="7"/>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Aceite para masajes con sensación de calor y sabor a ron, en frasco de 80 ml.</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>80 ml</t>
+        </is>
+      </c>
       <c r="Y171" t="inlineStr">
         <is>
           <t>sí</t>
@@ -17981,18 +18565,27 @@
         <f>IF(B171="","","productos/"&amp;B171&amp;"/")</f>
         <v>productos/ESZ-INT-120/</v>
       </c>
+      <c r="AG171" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="172" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A172" s="6" t="s">
-        <v>56</v>
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B172" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-121</t>
         </is>
       </c>
-      <c r="C172" s="6" t="s">
-        <v>1763</v>
+      <c r="C172" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo Euforia con CBD</t>
+        </is>
       </c>
       <c r="D172" s="10" t="s">
         <v>85</v>
@@ -18004,6 +18597,16 @@
         <v>12000</v>
       </c>
       <c r="I172" s="7"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Gel íntimo Sen Íntimo de la línea Multiorgasmos, versión Euforia con CBD, en sobre individual.</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y172" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18013,18 +18616,27 @@
         <f t="shared" ref="AC172:AC202" si="2">IF(B172="","","productos/"&amp;B172&amp;"/")</f>
         <v>productos/ESZ-INT-121/</v>
       </c>
+      <c r="AG172" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="173" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A173" s="6" t="s">
-        <v>56</v>
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B173" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-122</t>
         </is>
       </c>
-      <c r="C173" s="6" t="s">
-        <v>1765</v>
+      <c r="C173" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo Multiorgasmos frío</t>
+        </is>
       </c>
       <c r="D173" s="10" t="s">
         <v>85</v>
@@ -18036,6 +18648,16 @@
         <v>10000</v>
       </c>
       <c r="I173" s="7"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Gel íntimo Sen Íntimo de la línea Multiorgasmos con sensación fría, en sobre individual.</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y173" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18045,18 +18667,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-122/</v>
       </c>
+      <c r="AG173" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="174" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A174" s="6" t="s">
-        <v>56</v>
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B174" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-123</t>
         </is>
       </c>
-      <c r="C174" s="6" t="s">
-        <v>1767</v>
+      <c r="C174" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo lubricante caliente · Crema de whisky</t>
+        </is>
       </c>
       <c r="D174" s="10" t="s">
         <v>85</v>
@@ -18068,6 +18699,16 @@
         <v>10000</v>
       </c>
       <c r="I174" s="7"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Lubricante íntimo Sen Íntimo con sensación caliente y aroma a crema de whisky, en sobre individual.</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y174" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18077,18 +18718,27 @@
         <f>IF(#REF!="","","productos/"&amp;#REF!&amp;"/")</f>
         <v>productos/ESZ-INT-123/</v>
       </c>
+      <c r="AG174" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="175" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A175" s="6" t="s">
-        <v>56</v>
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B175" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-124</t>
         </is>
       </c>
-      <c r="C175" s="6" t="s">
-        <v>1769</v>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo lubricante Estrechante</t>
+        </is>
       </c>
       <c r="D175" s="10" t="s">
         <v>85</v>
@@ -18100,6 +18750,16 @@
         <v>12000</v>
       </c>
       <c r="I175" s="7"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Lubricante íntimo Sen Íntimo de la línea Estrechante, en sobre individual.</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y175" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18109,18 +18769,27 @@
         <f>IF(B174="","","productos/"&amp;B174&amp;"/")</f>
         <v>productos/ESZ-INT-124/</v>
       </c>
+      <c r="AG175" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="176" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A176" s="6" t="s">
-        <v>56</v>
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B176" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-125</t>
         </is>
       </c>
-      <c r="C176" s="6" t="s">
-        <v>1771</v>
+      <c r="C176" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo lubricante desensibilizante</t>
+        </is>
       </c>
       <c r="D176" s="10" t="s">
         <v>85</v>
@@ -18132,6 +18801,16 @@
         <v>10000</v>
       </c>
       <c r="I176" s="7"/>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Lubricante íntimo Sen Íntimo desensibilizante, en sobre individual. Lee las precauciones antes de usarlo.</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>Contiene un ingrediente desensibilizante: no lo uses para ocultar molestias. Si sientes dolor, detente. Prueba primero en una zona pequeña de la piel.</t>
+        </is>
+      </c>
       <c r="Y176" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18141,18 +18820,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-125/</v>
       </c>
+      <c r="AG176" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Los lubricantes desensibilizantes pueden ocultar dolor o lesiones. Recomiendo no publicarlo, o hacerlo solo con esta precaución.</t>
+        </is>
+      </c>
     </row>
     <row r="177" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A177" s="6" t="s">
-        <v>56</v>
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B177" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-126</t>
         </is>
       </c>
-      <c r="C177" s="6" t="s">
-        <v>1773</v>
+      <c r="C177" s="6" t="inlineStr">
+        <is>
+          <t>Sen Íntimo lubricante caliente · Caramelo</t>
+        </is>
       </c>
       <c r="D177" s="6" t="s">
         <v>85</v>
@@ -18164,6 +18852,16 @@
         <v>10000</v>
       </c>
       <c r="I177" s="7"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Lubricante íntimo Sen Íntimo con sensación caliente y aroma a caramelo, en sobre individual.</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y177" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18173,18 +18871,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-126/</v>
       </c>
+      <c r="AG177" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="178" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A178" s="6" t="s">
-        <v>56</v>
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B178" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-127</t>
         </is>
       </c>
-      <c r="C178" s="6" t="s">
-        <v>1775</v>
+      <c r="C178" s="6" t="inlineStr">
+        <is>
+          <t>Condones +SEX estimulantes x3</t>
+        </is>
       </c>
       <c r="D178" s="6" t="s">
         <v>85</v>
@@ -18196,6 +18903,21 @@
         <v>6000</v>
       </c>
       <c r="I178" s="7"/>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Condones +SEX estimulantes con sabor, en caja de 3 unidades.</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>Revisa la fecha de vencimiento y que el empaque esté intacto antes de usarlo.</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>3 unidades</t>
+        </is>
+      </c>
       <c r="Y178" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18205,18 +18927,27 @@
         <f>IF(B178="","","productos/"&amp;B178&amp;"/")</f>
         <v>productos/ESZ-INT-127/</v>
       </c>
+      <c r="AG178" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="179" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A179" s="6" t="s">
-        <v>56</v>
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B179" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-128</t>
         </is>
       </c>
-      <c r="C179" s="6" t="s">
-        <v>1777</v>
+      <c r="C179" s="6" t="inlineStr">
+        <is>
+          <t>Velas aromáticas Sen Íntimo x3</t>
+        </is>
       </c>
       <c r="D179" s="6" t="s">
         <v>85</v>
@@ -18228,6 +18959,21 @@
         <v>15000</v>
       </c>
       <c r="I179" s="7"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Set de 3 velas aromáticas Sen Íntimo para crear un ambiente cálido y relajado.</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>No dejes las velas encendidas sin supervisión.</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>3 unidades</t>
+        </is>
+      </c>
       <c r="Y179" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18237,18 +18983,27 @@
         <f>IF(B179="","","productos/"&amp;B179&amp;"/")</f>
         <v>productos/ESZ-INT-128/</v>
       </c>
+      <c r="AG179" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="180" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A180" s="6" t="s">
-        <v>56</v>
+      <c r="A180" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B180" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-129</t>
         </is>
       </c>
-      <c r="C180" s="6" t="s">
-        <v>1779</v>
+      <c r="C180" s="6" t="inlineStr">
+        <is>
+          <t>Aceite G-Hot caliente · Uva</t>
+        </is>
       </c>
       <c r="D180" s="6" t="s">
         <v>85</v>
@@ -18260,6 +19015,16 @@
         <v>20000</v>
       </c>
       <c r="I180" s="7"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Aceite artesanal G-Hot con sensación de calor y sabor a uva, en frasco pequeño fácil de llevar.</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y180" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18269,18 +19034,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-129/</v>
       </c>
+      <c r="AG180" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="181" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A181" s="6" t="s">
-        <v>56</v>
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B181" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-130</t>
         </is>
       </c>
-      <c r="C181" s="6" t="s">
-        <v>1780</v>
+      <c r="C181" s="6" t="inlineStr">
+        <is>
+          <t>Aceite G-Hot caliente · Piña colada</t>
+        </is>
       </c>
       <c r="D181" s="6" t="s">
         <v>85</v>
@@ -18292,6 +19066,16 @@
         <v>20000</v>
       </c>
       <c r="I181" s="7"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Aceite artesanal G-Hot con sensación de calor y sabor a piña colada, en frasco pequeño fácil de llevar.</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y181" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18301,18 +19085,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-130/</v>
       </c>
+      <c r="AG181" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="182" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A182" s="6" t="s">
-        <v>56</v>
+      <c r="A182" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B182" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-131</t>
         </is>
       </c>
-      <c r="C182" s="6" t="s">
-        <v>1783</v>
+      <c r="C182" s="6" t="inlineStr">
+        <is>
+          <t>Aceite G-Hot caliente · Halls</t>
+        </is>
       </c>
       <c r="D182" s="6" t="s">
         <v>85</v>
@@ -18324,6 +19117,16 @@
         <v>20000</v>
       </c>
       <c r="I182" s="7"/>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Aceite artesanal G-Hot con sensación de calor y sabor a menta tipo Halls, en frasco pequeño fácil de llevar.</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y182" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18333,18 +19136,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-131/</v>
       </c>
+      <c r="AG182" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="183" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A183" s="6" t="s">
-        <v>56</v>
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-132</t>
         </is>
       </c>
-      <c r="C183" s="6" t="s">
-        <v>1785</v>
+      <c r="C183" s="6" t="inlineStr">
+        <is>
+          <t>Aceite G-Hot caliente · Fresa con chocolate</t>
+        </is>
       </c>
       <c r="D183" s="6" t="s">
         <v>85</v>
@@ -18356,6 +19168,16 @@
         <v>20000</v>
       </c>
       <c r="I183" s="7"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Aceite artesanal G-Hot con sensación de calor y sabor a fresa con chocolate, en frasco pequeño fácil de llevar.</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
       <c r="Y183" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18365,18 +19187,27 @@
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-132/</v>
       </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+        </is>
+      </c>
     </row>
     <row r="184" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A184" s="6" t="s">
-        <v>56</v>
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>borrador</t>
+        </is>
       </c>
       <c r="B184" s="10" t="inlineStr">
         <is>
           <t>ESZ-INT-133</t>
         </is>
       </c>
-      <c r="C184" s="6" t="s">
-        <v>1787</v>
+      <c r="C184" s="6" t="inlineStr">
+        <is>
+          <t>Aceite caliente para masajes · Coco 30 ml</t>
+        </is>
       </c>
       <c r="D184" s="6" t="s">
         <v>85</v>
@@ -18388,6 +19219,21 @@
         <v>25000</v>
       </c>
       <c r="I184" s="7"/>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Aceite para masajes con sensación de calor y sabor a coco, en frasco de 30 ml.</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>Uso externo. Prueba primero en una zona pequeña de la piel y suspende su uso si notas irritación.</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
       <c r="Y184" t="inlineStr">
         <is>
           <t>sí</t>
@@ -18396,6 +19242,11 @@
       <c r="AC184" s="6" t="str">
         <f t="shared" si="2"/>
         <v>productos/ESZ-INT-133/</v>
+      </c>
+      <c r="AG184" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "oral" del nombre. El empaque de la foto no muestra el sabor coco: confírmalo.</t>
+        </is>
       </c>
     </row>
     <row r="185" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Publica 35 productos nuevos con foto (157 en total)
Pasa a "validado" 35 de los 39 productos con textos propuestos, por
indicación de Jorge y antes de la revisión de Diana (queda anotado en
notas_internas). Siguen en borrador: Shilajit (INT-105, empaque
contradictorio), Super Viga (INT-109, confirmar INVIMA), Ball Exotic
(INT-111, sin descripción) y el lubricante desensibilizante (INT-125).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/catalogo.xlsx
+++ b/catalogo/catalogo.xlsx
@@ -15883,7 +15883,7 @@
     <row r="120" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
@@ -15940,7 +15940,7 @@
       </c>
       <c r="AG120" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: ficha oficial https://skindrug.com.co/producto/sunface-aqua-antipigment/ y empaque. Aviso: El nombre del Excel decía "Aqua sin color"; el empaque y la ficha oficial dicen "Aqua Antipigment".</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: ficha oficial https://skindrug.com.co/producto/sunface-aqua-antipigment/ y empaque. Aviso: El nombre del Excel decía "Aqua sin color"; el empaque y la ficha oficial dicen "Aqua Antipigment".</t>
         </is>
       </c>
     </row>
@@ -16561,7 +16561,7 @@
     <row r="131" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="AG131" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: ficha oficial https://pharmaderm.com.co/producto/sunstop-oil-free-color/ y empaque. Aviso: Es el mismo producto que ESZ-PIE-001 (SunStop Oil Free Color, en borrador y sin precio). Conviene dejar solo uno.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: ficha oficial https://pharmaderm.com.co/producto/sunstop-oil-free-color/ y empaque. Aviso: Es el mismo producto que ESZ-PIE-001 (SunStop Oil Free Color, en borrador y sin precio). Conviene dejar solo uno.</t>
         </is>
       </c>
     </row>
@@ -16810,7 +16810,7 @@
     <row r="135" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
@@ -16852,14 +16852,14 @@
       </c>
       <c r="AG135" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="136" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B136" s="6" t="inlineStr">
@@ -16901,14 +16901,14 @@
       </c>
       <c r="AG136" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="137" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
@@ -16955,14 +16955,14 @@
       </c>
       <c r="AG137" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="138" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
@@ -17009,14 +17009,14 @@
       </c>
       <c r="AG138" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="139" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
@@ -17058,14 +17058,14 @@
       </c>
       <c r="AG139" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Hydaxer Hidratante colágeno"; el empaque dice "Hydraxer Face Oil Free · Hidratante facial" y no menciona colágeno.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Hydaxer Hidratante colágeno"; el empaque dice "Hydraxer Face Oil Free · Hidratante facial" y no menciona colágeno.</t>
         </is>
       </c>
     </row>
     <row r="140" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B140" s="6" t="inlineStr">
@@ -17107,14 +17107,14 @@
       </c>
       <c r="AG140" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="141" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
@@ -17156,14 +17156,14 @@
       </c>
       <c r="AG141" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="142" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
@@ -17210,14 +17210,14 @@
       </c>
       <c r="AG142" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet).</t>
         </is>
       </c>
     </row>
     <row r="143" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
@@ -17264,14 +17264,14 @@
       </c>
       <c r="AG143" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque y fichas de distribuidores autorizados de Sesderma.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque y fichas de distribuidores autorizados de Sesderma.</t>
         </is>
       </c>
     </row>
     <row r="144" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
@@ -17328,14 +17328,14 @@
       </c>
       <c r="AG144" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque y ficha técnica PLM https://www.medicamentosplm.com/Home/productos/cetopic_crema/83/101/51564/36.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque y ficha técnica PLM https://www.medicamentosplm.com/Home/productos/cetopic_crema/83/101/51564/36.</t>
         </is>
       </c>
     </row>
     <row r="145" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="AG145" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Ling-D"; el empaque dice "Lign-D".</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: texto del empaque (no se encontró ficha oficial en internet). Aviso: El Excel decía "Ling-D"; el empaque dice "Lign-D".</t>
         </is>
       </c>
     </row>
@@ -17797,7 +17797,7 @@
     <row r="157" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B157" s="6" t="inlineStr">
@@ -17846,14 +17846,14 @@
       </c>
       <c r="AG157" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="158" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B158" s="6" t="inlineStr">
@@ -17900,14 +17900,14 @@
       </c>
       <c r="AG158" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: El Excel decía "Hamboli"; el empaque dice "Hanboli".</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque. Aviso: El Excel decía "Hamboli"; el empaque dice "Hanboli".</t>
         </is>
       </c>
     </row>
     <row r="159" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B159" s="6" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="AG159" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "palpitante" del nombre: describe un efecto que no se puede verificar.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque. Aviso: Quité "palpitante" del nombre: describe un efecto que no se puede verificar.</t>
         </is>
       </c>
     </row>
@@ -18020,7 +18020,7 @@
     <row r="161" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B161" s="10" t="inlineStr">
@@ -18067,7 +18067,7 @@
       </c>
       <c r="AG161" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18123,7 @@
     <row r="163" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B163" s="6" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="AG163" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
@@ -18294,7 +18294,7 @@
     <row r="167" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B167" s="10" t="inlineStr">
@@ -18343,14 +18343,14 @@
       </c>
       <c r="AG167" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
         </is>
       </c>
     </row>
     <row r="168" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A168" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B168" s="10" t="inlineStr">
@@ -18399,14 +18399,14 @@
       </c>
       <c r="AG168" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque. Aviso: Quité "para sexo oral" del nombre (regla: nada explícito).</t>
         </is>
       </c>
     </row>
     <row r="169" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B169" s="10" t="inlineStr">
@@ -18455,14 +18455,14 @@
       </c>
       <c r="AG169" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="170" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B170" s="10" t="inlineStr">
@@ -18511,14 +18511,14 @@
       </c>
       <c r="AG170" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="171" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B171" s="10" t="inlineStr">
@@ -18567,14 +18567,14 @@
       </c>
       <c r="AG171" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="172" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B172" s="10" t="inlineStr">
@@ -18618,14 +18618,14 @@
       </c>
       <c r="AG172" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="173" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A173" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B173" s="10" t="inlineStr">
@@ -18669,14 +18669,14 @@
       </c>
       <c r="AG173" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="174" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A174" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B174" s="10" t="inlineStr">
@@ -18720,14 +18720,14 @@
       </c>
       <c r="AG174" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="175" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A175" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B175" s="10" t="inlineStr">
@@ -18771,7 +18771,7 @@
       </c>
       <c r="AG175" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
@@ -18829,7 +18829,7 @@
     <row r="177" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A177" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B177" s="10" t="inlineStr">
@@ -18873,14 +18873,14 @@
       </c>
       <c r="AG177" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="178" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A178" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B178" s="10" t="inlineStr">
@@ -18929,14 +18929,14 @@
       </c>
       <c r="AG178" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="179" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B179" s="10" t="inlineStr">
@@ -18985,14 +18985,14 @@
       </c>
       <c r="AG179" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="180" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B180" s="10" t="inlineStr">
@@ -19036,14 +19036,14 @@
       </c>
       <c r="AG180" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="181" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B181" s="10" t="inlineStr">
@@ -19087,14 +19087,14 @@
       </c>
       <c r="AG181" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="182" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B182" s="10" t="inlineStr">
@@ -19138,14 +19138,14 @@
       </c>
       <c r="AG182" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="183" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A183" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
@@ -19189,14 +19189,14 @@
       </c>
       <c r="AG183" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque.</t>
         </is>
       </c>
     </row>
     <row r="184" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A184" s="6" t="inlineStr">
         <is>
-          <t>borrador</t>
+          <t>validado</t>
         </is>
       </c>
       <c r="B184" s="10" t="inlineStr">
@@ -19245,7 +19245,7 @@
       </c>
       <c r="AG184" t="inlineStr">
         <is>
-          <t>[2026-10-28] Textos propuestos por Claude; pendientes de aprobación de Diana. Fuente: empaque. Aviso: Quité "oral" del nombre. El empaque de la foto no muestra el sabor coco: confírmalo.</t>
+          <t>[2026-10-28] Textos propuestos por Claude; publicados el 2026-10-28 por indicación de Jorge, antes de la revisión de Diana. Fuente: empaque. Aviso: Quité "oral" del nombre. El empaque de la foto no muestra el sabor coco: confírmalo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publica 4 suplementos de Equilibrio interno
Zarzaparrilla, Aceite de Orégano 6000 mg, Drenaje Linfático 60 y Ginseng
Royal Jelly x10: subcategoría Suplementos, descripción mínima (solo con el
nombre y, en el orégano, el texto del empaque), aviso de que no son
medicamentos y precauciones. Pendiente con Diana: registro INVIMA,
presentación e ingredientes, y fotos de tres de ellos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/catalogo.xlsx
+++ b/catalogo/catalogo.xlsx
@@ -17387,8 +17387,10 @@
       </c>
     </row>
     <row r="146" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A146" s="6" t="s">
-        <v>56</v>
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>validado</t>
+        </is>
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
@@ -17403,6 +17405,11 @@
       </c>
       <c r="E146" s="6" t="s">
         <v>1568</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
       </c>
       <c r="H146" s="9">
         <v>33000</v>
@@ -17411,10 +17418,25 @@
       <c r="J146" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Suplemento de zarzaparrilla de la marca Naturisol. No es un medicamento; consulta a un profesional de la salud antes de consumirlo.</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>No es un medicamento. No superes la dosis indicada en el empaque. Consulta a un profesional de la salud antes de consumirlo, sobre todo si estás en embarazo, lactancia o tomas medicamentos.</t>
+        </is>
+      </c>
       <c r="AC146" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-EQU-001/</v>
       </c>
+      <c r="AG146" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Descripción mínima redactada por Claude con el nombre del producto; publicada por indicación de Jorge. Pendiente con Diana: confirmar registro sanitario INVIMA, presentación e ingredientes..</t>
+        </is>
+      </c>
     </row>
     <row r="147" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6" t="s">
@@ -17489,22 +17511,31 @@
       </c>
     </row>
     <row r="149" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A149" s="6" t="s">
-        <v>56</v>
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>validado</t>
+        </is>
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
           <t>ESZ-EQU-004</t>
         </is>
       </c>
-      <c r="C149" s="6" t="s">
-        <v>1718</v>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>Aceite de Orégano 6000 mg</t>
+        </is>
       </c>
       <c r="D149" s="6" t="s">
         <v>85</v>
       </c>
       <c r="E149" s="6" t="s">
         <v>1568</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
       </c>
       <c r="H149" s="9">
         <v>45000</v>
@@ -17513,10 +17544,35 @@
       <c r="J149" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Aceite de orégano de 6.000 mg por porción con aceite de semilla negra, en 180 cápsulas blandas. Suplemento dietario, no es un medicamento.</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Aceite de orégano (alto en carvacrol) y aceite de semilla negra (timoquinona). Sin OGM, sin lácteos y sin gluten, según el empaque.</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>No es un medicamento. No superes la dosis indicada en el empaque. Consulta a un profesional de la salud antes de consumirlo, sobre todo si estás en embarazo, lactancia o tomas medicamentos.</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>180 cápsulas blandas</t>
+        </is>
+      </c>
       <c r="AC149" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-EQU-004/</v>
       </c>
+      <c r="AG149" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Descripción mínima redactada por Claude con el nombre del producto y el texto del empaque; publicada por indicación de Jorge. Pendiente con Diana: confirmar registro sanitario INVIMA, presentación e ingredientes..</t>
+        </is>
+      </c>
     </row>
     <row r="150" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A150" s="6" t="s">
@@ -17586,8 +17642,10 @@
       </c>
     </row>
     <row r="152" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A152" s="6" t="s">
-        <v>56</v>
+      <c r="A152" s="6" t="inlineStr">
+        <is>
+          <t>validado</t>
+        </is>
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
@@ -17602,6 +17660,11 @@
       </c>
       <c r="E152" s="6" t="s">
         <v>1568</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
       </c>
       <c r="H152" s="9">
         <v>60000</v>
@@ -17610,14 +17673,31 @@
       <c r="J152" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Suplemento Drenaje Linfático 60. No es un medicamento; consulta a un profesional de la salud antes de consumirlo.</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>No es un medicamento. No superes la dosis indicada en el empaque. Consulta a un profesional de la salud antes de consumirlo, sobre todo si estás en embarazo, lactancia o tomas medicamentos.</t>
+        </is>
+      </c>
       <c r="AC152" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-EQU-007/</v>
       </c>
+      <c r="AG152" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Descripción mínima redactada por Claude con el nombre del producto; publicada por indicación de Jorge. Pendiente con Diana: confirmar registro sanitario INVIMA, presentación e ingredientes..</t>
+        </is>
+      </c>
     </row>
     <row r="153" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A153" s="6" t="s">
-        <v>56</v>
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>validado</t>
+        </is>
       </c>
       <c r="B153" s="6" t="inlineStr">
         <is>
@@ -17632,6 +17712,11 @@
       </c>
       <c r="E153" s="6" t="s">
         <v>1568</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
       </c>
       <c r="H153" s="9">
         <v>65000</v>
@@ -17640,9 +17725,29 @@
       <c r="J153" s="6" t="s">
         <v>63</v>
       </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Bebible de ginseng y jalea real en caja de 10 unidades. Es un suplemento, no un medicamento; consulta a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>No es un medicamento. No superes la dosis indicada en el empaque. Consulta a un profesional de la salud antes de consumirlo, sobre todo si estás en embarazo, lactancia o tomas medicamentos.</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>Caja de 10 bebibles</t>
+        </is>
+      </c>
       <c r="AC153" s="6" t="str">
         <f t="shared" si="1"/>
         <v>productos/ESZ-EQU-008/</v>
+      </c>
+      <c r="AG153" t="inlineStr">
+        <is>
+          <t>[2026-10-28] Descripción mínima redactada por Claude con el nombre del producto; publicada por indicación de Jorge. Pendiente con Diana: confirmar registro sanitario INVIMA, presentación e ingredientes..</t>
+        </is>
       </c>
     </row>
     <row r="154" spans="1:29" s="6" customFormat="1" ht="29" x14ac:dyDescent="0.35">

</xml_diff>